<commit_message>
Added Basic Items to Product Backlog
Added some basic items to the product backlog. Further additions and modifications will likely need to be made.
</commit_message>
<xml_diff>
--- a/MealPlanner/sprints/Product Backlog.xlsx
+++ b/MealPlanner/sprints/Product Backlog.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22325"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29721"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonathan Corley\git\SE2-project-repos-sample\sprints\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04EC7C4E-5288-43E2-BCCD-AFE8A3B4E981}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{629A70E1-1343-4586-A1FC-974210C1FC10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="39780" yWindow="1380" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
   <si>
     <t>Priority</t>
   </si>
@@ -39,20 +50,128 @@
     <t>Why</t>
   </si>
   <si>
-    <t>As a…</t>
-  </si>
-  <si>
-    <t>I want…</t>
-  </si>
-  <si>
-    <t>So that…</t>
+    <t>As a user.</t>
+  </si>
+  <si>
+    <t>I want to login.</t>
+  </si>
+  <si>
+    <t>So that I can access the system.</t>
+  </si>
+  <si>
+    <t>I want to create an account.</t>
+  </si>
+  <si>
+    <t>So that I can login.</t>
+  </si>
+  <si>
+    <t>I want to make meals.</t>
+  </si>
+  <si>
+    <t>So that I can add them to the planner.</t>
+  </si>
+  <si>
+    <t>I want to add ingredents to the planner.</t>
+  </si>
+  <si>
+    <t>So that I can plan items outside of meals.</t>
+  </si>
+  <si>
+    <t>I want to add meals to the planner.</t>
+  </si>
+  <si>
+    <t>So that I can keep track of my meals.</t>
+  </si>
+  <si>
+    <t>I want to view my planner.</t>
+  </si>
+  <si>
+    <t>So that I know which food items I have planned.</t>
+  </si>
+  <si>
+    <t>I want to delete meals.</t>
+  </si>
+  <si>
+    <t>So that clear meals that I don't intend to plan.</t>
+  </si>
+  <si>
+    <t>I want to filter ingredients alphabetically.</t>
+  </si>
+  <si>
+    <t>So that I can more easily find the ingredients I want to add.</t>
+  </si>
+  <si>
+    <t>I want to remove ingredients from the planner.</t>
+  </si>
+  <si>
+    <t>So that I can get rid indivisual items I no longer want.</t>
+  </si>
+  <si>
+    <t>I want to remove meals from the planner.</t>
+  </si>
+  <si>
+    <t>So that I can get rid of meals I no longer wish to prepare.</t>
+  </si>
+  <si>
+    <t>I want to generate a grocery list.</t>
+  </si>
+  <si>
+    <t>So that I know what to buy for what I had planned.</t>
+  </si>
+  <si>
+    <t>I want to make meals recurring.</t>
+  </si>
+  <si>
+    <t>So that I don't need to repeatedly add them.</t>
+  </si>
+  <si>
+    <t>I want to add descriptions to meals.</t>
+  </si>
+  <si>
+    <t>So that I can keep track of additional information about the meal.</t>
+  </si>
+  <si>
+    <t>I want to modifiy the grocery list.</t>
+  </si>
+  <si>
+    <t>So that I can keep track of which items I have and what I still need.</t>
+  </si>
+  <si>
+    <t>I want to filter ingredients by nutritional content.</t>
+  </si>
+  <si>
+    <t>So that I can find ingredients that fit my nutritional needs.</t>
+  </si>
+  <si>
+    <t>I want to filter meals by nutritional content.</t>
+  </si>
+  <si>
+    <t>So that I can find meals that fit my nutritional needs.</t>
+  </si>
+  <si>
+    <t>I want to see a summary of nutritional information for foods planned.</t>
+  </si>
+  <si>
+    <t>So that I can quickly assess if what I have planned fits my needs.</t>
+  </si>
+  <si>
+    <t>I want to add notes to days on the planner.</t>
+  </si>
+  <si>
+    <t>So that I can store important information regarding what I had planned that day.</t>
+  </si>
+  <si>
+    <t>I want to modifiy notes on days on the planner.</t>
+  </si>
+  <si>
+    <t>So that I can update the information as my needs and plans change.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,9 +206,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -370,15 +492,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="13.5703125" customWidth="1"/>
     <col min="3" max="3" width="37.5703125" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -392,7 +514,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="30.75">
       <c r="A2">
         <v>1</v>
       </c>
@@ -402,11 +524,266 @@
       <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
+    <row r="3" spans="1:4">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="30.75">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30.75">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="30.75">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="30.75">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="30.75">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="45.75">
+      <c r="A9">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="45.75">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="30.75">
+      <c r="A11">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="30.75">
+      <c r="A12">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="30.75">
+      <c r="A13">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="45.75">
+      <c r="A14">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="45.75">
+      <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="30.75">
+      <c r="A16">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="30.75">
+      <c r="A17">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="45.75">
+      <c r="A18">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="45.75">
+      <c r="A19">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="45.75">
+      <c r="A20">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D20">
+    <sortCondition ref="A2:A20"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>